<commit_message>
Completed Milestone 3 business logic and integration testing
</commit_message>
<xml_diff>
--- a/Bussiness_Logic/generated_reports/Instructor_Summary.xlsx
+++ b/Bussiness_Logic/generated_reports/Instructor_Summary.xlsx
@@ -450,13 +450,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" t="n">
-        <v>75.22</v>
+        <v>71.03</v>
       </c>
       <c r="D2" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>

</xml_diff>